<commit_message>
Add visual insights dashboard to trend workbook
</commit_message>
<xml_diff>
--- a/outputs/019fcf4b-cafe-75c0-814f-d0b3e093c2ac/trend-meme-stock-cases.xlsx
+++ b/outputs/019fcf4b-cafe-75c0-814f-d0b3e093c2ac/trend-meme-stock-cases.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_안내" sheetId="1" r:id="Rb4ebd207e3114429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_유행이벤트" sheetId="2" r:id="Raf14ee8c128a4edf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_종목반응" sheetId="3" r:id="Rded66f7fccea48f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_출처" sheetId="4" r:id="R67ceea24a0454ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_판정기준" sheetId="5" r:id="Rbf1f818408064f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_안내" sheetId="1" r:id="R2a1c0cdb9f8c45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_유행이벤트" sheetId="2" r:id="R5de175dda10947f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_종목반응" sheetId="3" r:id="R3c950a999df740f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_출처" sheetId="4" r:id="R19a806caaa15442c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_판정기준" sheetId="5" r:id="Rd7a186bd37664a64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,12 +17,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="@"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="25">
+  <x:fonts count="33">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -169,8 +171,54 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17213C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5C667A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF5C667A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF157A5A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FFA65D00"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFA65D00"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="48">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -277,8 +325,138 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071A52"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF1FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4006D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163D8C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6C3BE8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23A8E0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF157A5A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F8F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA65D00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071A52"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF1FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4006D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163D8C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF6C3BE8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23A8E0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF157A5A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F8F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA65D00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF5D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="20">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -362,11 +540,93 @@
         <x:color rgb="FFD7DEEC"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7DEEC"/>
+      </x:right>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="184">
+  <x:cellXfs count="781">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -810,6 +1070,1271 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="24" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="25" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="26" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="27" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="27" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="28" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="28" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="29" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="30" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="23" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="31" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="25" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="13" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="37" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="37" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="28" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="39" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="39" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="40" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="40" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="41" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="41" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="42" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="26" fillId="42" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="26" fillId="42" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="43" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="36" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="44" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="39" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="30" fillId="39" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="25" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="13" fillId="45" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="47" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="32" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -911,6 +2436,620 @@
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="975"/>
+              <a:t>연도별 유행·트렌드 사건 수</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="975"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>사건 수</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="F4006D"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'00_안내'!$A$49:$A$66</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'00_안내'!$B$49:$B$66</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="600"/>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="30"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="975"/>
+              <a:t>대분류별 사건 수</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="975"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>전체 사건</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="163D8C"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'00_안내'!$D$49:$D$57</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'00_안내'!$E$49:$E$57</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="675"/>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="100"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="975"/>
+              <a:t>주가 연결 상태 — 70건 확인, 228건 조사 후보</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="975"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:doughnutChart>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>사건 수</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'00_안내'!$I$49:$I$50</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'00_안내'!$J$49:$J$50</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+      </c:doughnutChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="975"/>
+              <a:t>대분류별 주가 연결률 — 표본 크기 유의</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="975"/>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>주가 연결률</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="6C3BE8"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'00_안내'!$K$49:$K$57</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'00_안내'!$L$49:$L$57</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="675"/>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3c1b4ec7a44d43d7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb476cb21c70844bd"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26224abf435c4ec9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1ec5a1962078468f"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1142,405 +3281,1601 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="11" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="11" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="11" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="11" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="94" t="str">
-        <x:v>키움 트렌드 인사이트 — 2009~2026 비정치 유행·밈·트렌드 원장</x:v>
-      </x:c>
-      <x:c r="B1"/>
-      <x:c r="C1"/>
-      <x:c r="D1"/>
-      <x:c r="E1"/>
-      <x:c r="F1"/>
-      <x:c r="G1"/>
-      <x:c r="H1"/>
-      <x:c r="I1"/>
-      <x:c r="J1"/>
-    </x:row>
-    <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="98" t="str">
-        <x:v>최신 연도부터 확인하고, 같은 연도 안에서는 표준 대분류·소분류로 탐색합니다. 주가 연결 여부와 무관하게 유행 사실을 먼저 축적하며 정치 테마는 제외합니다.</x:v>
-      </x:c>
-      <x:c r="B2" s="98"/>
-      <x:c r="C2" s="98"/>
-      <x:c r="D2" s="98"/>
-      <x:c r="E2" s="98"/>
-      <x:c r="F2" s="98"/>
-      <x:c r="G2" s="98"/>
-      <x:c r="H2" s="98"/>
-      <x:c r="I2" s="98"/>
-      <x:c r="J2" s="98"/>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="484" t="str">
+        <x:v>키움 트렌드 인사이트 — 데이터 한눈에 보기</x:v>
+      </x:c>
+      <x:c r="B1" s="484"/>
+      <x:c r="C1" s="484"/>
+      <x:c r="D1" s="484"/>
+      <x:c r="E1" s="484"/>
+      <x:c r="F1" s="484"/>
+      <x:c r="G1" s="484"/>
+      <x:c r="H1" s="484"/>
+      <x:c r="I1" s="484"/>
+      <x:c r="J1" s="484"/>
+      <x:c r="K1" s="484"/>
+      <x:c r="L1" s="484"/>
+      <x:c r="M1" s="484"/>
+      <x:c r="N1" s="484"/>
+      <x:c r="O1" s="484"/>
+      <x:c r="P1" s="484"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="488" t="str">
+        <x:v>2009~2026년 비정치 인터넷·SNS 유행 298건을 연도·카테고리·주가 연결 상태로 요약했습니다. 유행은 매수 신호가 아니라 기업 조사의 출발점입니다.</x:v>
+      </x:c>
+      <x:c r="B2" s="488"/>
+      <x:c r="C2" s="488"/>
+      <x:c r="D2" s="488"/>
+      <x:c r="E2" s="488"/>
+      <x:c r="F2" s="488"/>
+      <x:c r="G2" s="488"/>
+      <x:c r="H2" s="488"/>
+      <x:c r="I2" s="488"/>
+      <x:c r="J2" s="488"/>
+      <x:c r="K2" s="488"/>
+      <x:c r="L2" s="488"/>
+      <x:c r="M2" s="488"/>
+      <x:c r="N2" s="488"/>
+      <x:c r="O2" s="488"/>
+      <x:c r="P2" s="488"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="194" t="str">
+        <x:v>읽는 순서  ① 핵심 숫자 → ② 데이터가 말하는 세 가지 → ③ 연도·카테고리 분포 → ④ 주가 연결 정도</x:v>
+      </x:c>
+      <x:c r="B3" s="194"/>
+      <x:c r="C3" s="194"/>
+      <x:c r="D3" s="194"/>
+      <x:c r="E3" s="194"/>
+      <x:c r="F3" s="194"/>
+      <x:c r="G3" s="194"/>
+      <x:c r="H3" s="194"/>
+      <x:c r="I3" s="194"/>
+      <x:c r="J3" s="194"/>
+      <x:c r="K3" s="194"/>
+      <x:c r="L3" s="194"/>
+      <x:c r="M3" s="194"/>
+      <x:c r="N3" s="194"/>
+      <x:c r="O3" s="194"/>
+      <x:c r="P3" s="194"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="102" t="str">
-        <x:v>유행 사건</x:v>
-      </x:c>
-      <x:c r="B4" s="104" t="n">
+      <x:c r="A4" s="184"/>
+      <x:c r="B4" s="184"/>
+      <x:c r="C4" s="184"/>
+      <x:c r="D4" s="184"/>
+      <x:c r="E4" s="184"/>
+      <x:c r="F4" s="184"/>
+      <x:c r="G4" s="184"/>
+      <x:c r="H4" s="184"/>
+      <x:c r="I4" s="184"/>
+      <x:c r="J4" s="184"/>
+      <x:c r="K4" s="184"/>
+      <x:c r="L4" s="184"/>
+      <x:c r="M4" s="184"/>
+      <x:c r="N4" s="184"/>
+      <x:c r="O4" s="184"/>
+      <x:c r="P4" s="184"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="496" t="str">
+        <x:v>전체 유행 사건</x:v>
+      </x:c>
+      <x:c r="B5" s="497"/>
+      <x:c r="C5" s="498"/>
+      <x:c r="D5" s="496" t="str">
+        <x:v>주가 반응 확인</x:v>
+      </x:c>
+      <x:c r="E5" s="497"/>
+      <x:c r="F5" s="498"/>
+      <x:c r="G5" s="496" t="str">
+        <x:v>후속 조사 후보</x:v>
+      </x:c>
+      <x:c r="H5" s="497"/>
+      <x:c r="I5" s="498"/>
+      <x:c r="J5" s="496" t="str">
+        <x:v>가장 큰 카테고리</x:v>
+      </x:c>
+      <x:c r="K5" s="497"/>
+      <x:c r="L5" s="498"/>
+      <x:c r="M5" s="496" t="str">
+        <x:v>가장 많은 연도</x:v>
+      </x:c>
+      <x:c r="N5" s="497"/>
+      <x:c r="O5" s="497"/>
+      <x:c r="P5" s="498"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="519" t="n">
         <x:f>COUNTA('01_유행이벤트'!$A$6:$A$303)</x:f>
         <x:v>298</x:v>
       </x:c>
-      <x:c r="C4" s="102" t="str">
-        <x:v>주가 연결 사건</x:v>
-      </x:c>
-      <x:c r="D4" s="104" t="n">
+      <x:c r="B6" s="520"/>
+      <x:c r="C6" s="521"/>
+      <x:c r="D6" s="559" t="n">
         <x:f>COUNTIF('01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
         <x:v>70</x:v>
       </x:c>
-      <x:c r="E4" s="102" t="str">
-        <x:v>주가 미연결·미확인</x:v>
-      </x:c>
-      <x:c r="F4" s="104" t="n">
+      <x:c r="E6" s="560"/>
+      <x:c r="F6" s="561"/>
+      <x:c r="G6" s="585" t="n">
         <x:f>COUNTIF('01_유행이벤트'!$I$6:$I$303,"주가 미확인·연결 전")</x:f>
         <x:v>228</x:v>
       </x:c>
-      <x:c r="G4" s="102" t="str">
-        <x:v>종목 반응 행</x:v>
-      </x:c>
-      <x:c r="H4" s="104" t="n">
-        <x:f>COUNTA('02_종목반응'!$A$6:$A$166)</x:f>
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="I4" s="102" t="str">
-        <x:v>출처</x:v>
-      </x:c>
-      <x:c r="J4" s="104" t="n">
-        <x:f>COUNTA('03_출처'!$A$5:$A$136)</x:f>
-        <x:v>132</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="107" t="str">
-        <x:v>원장 구성</x:v>
-      </x:c>
-      <x:c r="B6" s="107"/>
-      <x:c r="C6" s="107"/>
-      <x:c r="D6" s="107"/>
-      <x:c r="E6" s="107"/>
-      <x:c r="F6" s="107" t="str">
-        <x:v>해석 원칙</x:v>
-      </x:c>
-      <x:c r="G6" s="107"/>
-      <x:c r="H6" s="107"/>
-      <x:c r="I6" s="107"/>
-      <x:c r="J6" s="107"/>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="113" t="str">
-        <x:v>01 유행이벤트</x:v>
-      </x:c>
-      <x:c r="B7" s="111" t="str">
-        <x:v>연도 내림차순 → 대분류 → 소분류 → 사건명</x:v>
-      </x:c>
-      <x:c r="C7" s="111"/>
-      <x:c r="D7" s="111"/>
-      <x:c r="E7" s="111"/>
-      <x:c r="F7" s="116" t="str">
+      <x:c r="H6" s="586"/>
+      <x:c r="I6" s="587"/>
+      <x:c r="J6" s="611" t="str">
+        <x:f>INDEX($D$49:$D$57,MATCH(MAX($E$49:$E$57),$E$49:$E$57,0))</x:f>
+        <x:v>콘텐츠·엔터</x:v>
+      </x:c>
+      <x:c r="K6" s="612"/>
+      <x:c r="L6" s="613"/>
+      <x:c r="M6" s="643" t="n">
+        <x:f>INDEX($A$49:$A$66,MATCH(MAX($B$49:$B$66),$B$49:$B$66,0))</x:f>
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="N6" s="644"/>
+      <x:c r="O6" s="644"/>
+      <x:c r="P6" s="645"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="522"/>
+      <x:c r="B7" s="523"/>
+      <x:c r="C7" s="524"/>
+      <x:c r="D7" s="562"/>
+      <x:c r="E7" s="563"/>
+      <x:c r="F7" s="564"/>
+      <x:c r="G7" s="588"/>
+      <x:c r="H7" s="589"/>
+      <x:c r="I7" s="590"/>
+      <x:c r="J7" s="614"/>
+      <x:c r="K7" s="615"/>
+      <x:c r="L7" s="616"/>
+      <x:c r="M7" s="646"/>
+      <x:c r="N7" s="647"/>
+      <x:c r="O7" s="647"/>
+      <x:c r="P7" s="648"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="536" t="str">
+        <x:f>"2009~2026 · 출처 "&amp;COUNTA('03_출처'!$A$5:$A$136)&amp;"개"</x:f>
+        <x:v>2009~2026 · 출처 132개</x:v>
+      </x:c>
+      <x:c r="B8" s="537"/>
+      <x:c r="C8" s="538"/>
+      <x:c r="D8" s="536" t="str">
+        <x:f>"전체의 "&amp;TEXT(D6/A6,"0.0%")</x:f>
+        <x:v>전체의 23.5%</x:v>
+      </x:c>
+      <x:c r="E8" s="537"/>
+      <x:c r="F8" s="538"/>
+      <x:c r="G8" s="536" t="str">
+        <x:f>"전체의 "&amp;TEXT(G6/A6,"0.0%")</x:f>
+        <x:v>전체의 76.5%</x:v>
+      </x:c>
+      <x:c r="H8" s="537"/>
+      <x:c r="I8" s="538"/>
+      <x:c r="J8" s="536" t="str">
+        <x:f>MAX($E$49:$E$57)&amp;"건 · "&amp;TEXT(MAX($E$49:$E$57)/A6,"0.0%")</x:f>
+        <x:v>89건 · 29.9%</x:v>
+      </x:c>
+      <x:c r="K8" s="537"/>
+      <x:c r="L8" s="538"/>
+      <x:c r="M8" s="536" t="str">
+        <x:f>MAX($B$49:$B$66)&amp;"건 · 2026년은 진행 중"</x:f>
+        <x:v>27건 · 2026년은 진행 중</x:v>
+      </x:c>
+      <x:c r="N8" s="537"/>
+      <x:c r="O8" s="537"/>
+      <x:c r="P8" s="538"/>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="184"/>
+      <x:c r="B9" s="184"/>
+      <x:c r="C9" s="184"/>
+      <x:c r="D9" s="184"/>
+      <x:c r="E9" s="184"/>
+      <x:c r="F9" s="184"/>
+      <x:c r="G9" s="184"/>
+      <x:c r="H9" s="184"/>
+      <x:c r="I9" s="184"/>
+      <x:c r="J9" s="184"/>
+      <x:c r="K9" s="184"/>
+      <x:c r="L9" s="184"/>
+      <x:c r="M9" s="184"/>
+      <x:c r="N9" s="184"/>
+      <x:c r="O9" s="184"/>
+      <x:c r="P9" s="184"/>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="651" t="str">
+        <x:v>데이터가 말하는 세 가지</x:v>
+      </x:c>
+      <x:c r="B10" s="651"/>
+      <x:c r="C10" s="651"/>
+      <x:c r="D10" s="651"/>
+      <x:c r="E10" s="651"/>
+      <x:c r="F10" s="651"/>
+      <x:c r="G10" s="651"/>
+      <x:c r="H10" s="651"/>
+      <x:c r="I10" s="651"/>
+      <x:c r="J10" s="651"/>
+      <x:c r="K10" s="651"/>
+      <x:c r="L10" s="651"/>
+      <x:c r="M10" s="651"/>
+      <x:c r="N10" s="651"/>
+      <x:c r="O10" s="651"/>
+      <x:c r="P10" s="651"/>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="672" t="str">
+        <x:f>"① 콘텐츠·엔터 "&amp;E49&amp;"건 + 식품·음료 "&amp;E50&amp;"건 = 전체 "&amp;TEXT((E49+E50)/A6,"0.0%")</x:f>
+        <x:v>① 콘텐츠·엔터 89건 + 식품·음료 76건 = 전체 55.4%</x:v>
+      </x:c>
+      <x:c r="B11" s="673"/>
+      <x:c r="C11" s="673"/>
+      <x:c r="D11" s="673"/>
+      <x:c r="E11" s="674"/>
+      <x:c r="F11" s="697" t="str">
+        <x:f>"② 주가 반응 확인 "&amp;D6&amp;"건보다 조사 대기 "&amp;G6&amp;"건이 "&amp;TEXT(G6/D6,"0.0x")&amp;" 많음"</x:f>
+        <x:v>② 주가 반응 확인 70건보다 조사 대기 228건이 3.3x 많음</x:v>
+      </x:c>
+      <x:c r="G11" s="698"/>
+      <x:c r="H11" s="698"/>
+      <x:c r="I11" s="698"/>
+      <x:c r="J11" s="699"/>
+      <x:c r="K11" s="723" t="str">
+        <x:f>"③ 최다 기록 연도 "&amp;M6&amp;"년 "&amp;MAX($B$49:$B$66)&amp;"건 · 최근 기록 집중"</x:f>
+        <x:v>③ 최다 기록 연도 2023년 27건 · 최근 기록 집중</x:v>
+      </x:c>
+      <x:c r="L11" s="724"/>
+      <x:c r="M11" s="724"/>
+      <x:c r="N11" s="724"/>
+      <x:c r="O11" s="724"/>
+      <x:c r="P11" s="725"/>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="675"/>
+      <x:c r="B12" s="676"/>
+      <x:c r="C12" s="676"/>
+      <x:c r="D12" s="676"/>
+      <x:c r="E12" s="677"/>
+      <x:c r="F12" s="700"/>
+      <x:c r="G12" s="701"/>
+      <x:c r="H12" s="701"/>
+      <x:c r="I12" s="701"/>
+      <x:c r="J12" s="702"/>
+      <x:c r="K12" s="726"/>
+      <x:c r="L12" s="727"/>
+      <x:c r="M12" s="727"/>
+      <x:c r="N12" s="727"/>
+      <x:c r="O12" s="727"/>
+      <x:c r="P12" s="728"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="184"/>
+      <x:c r="B13" s="184"/>
+      <x:c r="C13" s="184"/>
+      <x:c r="D13" s="184"/>
+      <x:c r="E13" s="184"/>
+      <x:c r="F13" s="184"/>
+      <x:c r="G13" s="184"/>
+      <x:c r="H13" s="184"/>
+      <x:c r="I13" s="184"/>
+      <x:c r="J13" s="184"/>
+      <x:c r="K13" s="184"/>
+      <x:c r="L13" s="184"/>
+      <x:c r="M13" s="184"/>
+      <x:c r="N13" s="184"/>
+      <x:c r="O13" s="184"/>
+      <x:c r="P13" s="184"/>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="184"/>
+      <x:c r="B14" s="184"/>
+      <x:c r="C14" s="184"/>
+      <x:c r="D14" s="184"/>
+      <x:c r="E14" s="184"/>
+      <x:c r="F14" s="184"/>
+      <x:c r="G14" s="184"/>
+      <x:c r="H14" s="184"/>
+      <x:c r="I14" s="184"/>
+      <x:c r="J14" s="184"/>
+      <x:c r="K14" s="184"/>
+      <x:c r="L14" s="184"/>
+      <x:c r="M14" s="184"/>
+      <x:c r="N14" s="184"/>
+      <x:c r="O14" s="184"/>
+      <x:c r="P14" s="184"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="184"/>
+      <x:c r="B15" s="184"/>
+      <x:c r="C15" s="184"/>
+      <x:c r="D15" s="184"/>
+      <x:c r="E15" s="184"/>
+      <x:c r="F15" s="184"/>
+      <x:c r="G15" s="184"/>
+      <x:c r="H15" s="184"/>
+      <x:c r="I15" s="184"/>
+      <x:c r="J15" s="184"/>
+      <x:c r="K15" s="184"/>
+      <x:c r="L15" s="184"/>
+      <x:c r="M15" s="184"/>
+      <x:c r="N15" s="184"/>
+      <x:c r="O15" s="184"/>
+      <x:c r="P15" s="184"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="184"/>
+      <x:c r="B16" s="184"/>
+      <x:c r="C16" s="184"/>
+      <x:c r="D16" s="184"/>
+      <x:c r="E16" s="184"/>
+      <x:c r="F16" s="184"/>
+      <x:c r="G16" s="184"/>
+      <x:c r="H16" s="184"/>
+      <x:c r="I16" s="184"/>
+      <x:c r="J16" s="184"/>
+      <x:c r="K16" s="184"/>
+      <x:c r="L16" s="184"/>
+      <x:c r="M16" s="184"/>
+      <x:c r="N16" s="184"/>
+      <x:c r="O16" s="184"/>
+      <x:c r="P16" s="184"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="184"/>
+      <x:c r="B17" s="184"/>
+      <x:c r="C17" s="184"/>
+      <x:c r="D17" s="184"/>
+      <x:c r="E17" s="184"/>
+      <x:c r="F17" s="184"/>
+      <x:c r="G17" s="184"/>
+      <x:c r="H17" s="184"/>
+      <x:c r="I17" s="184"/>
+      <x:c r="J17" s="184"/>
+      <x:c r="K17" s="184"/>
+      <x:c r="L17" s="184"/>
+      <x:c r="M17" s="184"/>
+      <x:c r="N17" s="184"/>
+      <x:c r="O17" s="184"/>
+      <x:c r="P17" s="184"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="184"/>
+      <x:c r="B18" s="184"/>
+      <x:c r="C18" s="184"/>
+      <x:c r="D18" s="184"/>
+      <x:c r="E18" s="184"/>
+      <x:c r="F18" s="184"/>
+      <x:c r="G18" s="184"/>
+      <x:c r="H18" s="184"/>
+      <x:c r="I18" s="184"/>
+      <x:c r="J18" s="184"/>
+      <x:c r="K18" s="184"/>
+      <x:c r="L18" s="184"/>
+      <x:c r="M18" s="184"/>
+      <x:c r="N18" s="184"/>
+      <x:c r="O18" s="184"/>
+      <x:c r="P18" s="184"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="184"/>
+      <x:c r="B19" s="184"/>
+      <x:c r="C19" s="184"/>
+      <x:c r="D19" s="184"/>
+      <x:c r="E19" s="184"/>
+      <x:c r="F19" s="184"/>
+      <x:c r="G19" s="184"/>
+      <x:c r="H19" s="184"/>
+      <x:c r="I19" s="184"/>
+      <x:c r="J19" s="184"/>
+      <x:c r="K19" s="184"/>
+      <x:c r="L19" s="184"/>
+      <x:c r="M19" s="184"/>
+      <x:c r="N19" s="184"/>
+      <x:c r="O19" s="184"/>
+      <x:c r="P19" s="184"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="184"/>
+      <x:c r="B20" s="184"/>
+      <x:c r="C20" s="184"/>
+      <x:c r="D20" s="184"/>
+      <x:c r="E20" s="184"/>
+      <x:c r="F20" s="184"/>
+      <x:c r="G20" s="184"/>
+      <x:c r="H20" s="184"/>
+      <x:c r="I20" s="184"/>
+      <x:c r="J20" s="184"/>
+      <x:c r="K20" s="184"/>
+      <x:c r="L20" s="184"/>
+      <x:c r="M20" s="184"/>
+      <x:c r="N20" s="184"/>
+      <x:c r="O20" s="184"/>
+      <x:c r="P20" s="184"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="184"/>
+      <x:c r="B21" s="184"/>
+      <x:c r="C21" s="184"/>
+      <x:c r="D21" s="184"/>
+      <x:c r="E21" s="184"/>
+      <x:c r="F21" s="184"/>
+      <x:c r="G21" s="184"/>
+      <x:c r="H21" s="184"/>
+      <x:c r="I21" s="184"/>
+      <x:c r="J21" s="184"/>
+      <x:c r="K21" s="184"/>
+      <x:c r="L21" s="184"/>
+      <x:c r="M21" s="184"/>
+      <x:c r="N21" s="184"/>
+      <x:c r="O21" s="184"/>
+      <x:c r="P21" s="184"/>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="184"/>
+      <x:c r="B22" s="184"/>
+      <x:c r="C22" s="184"/>
+      <x:c r="D22" s="184"/>
+      <x:c r="E22" s="184"/>
+      <x:c r="F22" s="184"/>
+      <x:c r="G22" s="184"/>
+      <x:c r="H22" s="184"/>
+      <x:c r="I22" s="184"/>
+      <x:c r="J22" s="184"/>
+      <x:c r="K22" s="184"/>
+      <x:c r="L22" s="184"/>
+      <x:c r="M22" s="184"/>
+      <x:c r="N22" s="184"/>
+      <x:c r="O22" s="184"/>
+      <x:c r="P22" s="184"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="184"/>
+      <x:c r="B23" s="184"/>
+      <x:c r="C23" s="184"/>
+      <x:c r="D23" s="184"/>
+      <x:c r="E23" s="184"/>
+      <x:c r="F23" s="184"/>
+      <x:c r="G23" s="184"/>
+      <x:c r="H23" s="184"/>
+      <x:c r="I23" s="184"/>
+      <x:c r="J23" s="184"/>
+      <x:c r="K23" s="184"/>
+      <x:c r="L23" s="184"/>
+      <x:c r="M23" s="184"/>
+      <x:c r="N23" s="184"/>
+      <x:c r="O23" s="184"/>
+      <x:c r="P23" s="184"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="184"/>
+      <x:c r="B24" s="184"/>
+      <x:c r="C24" s="184"/>
+      <x:c r="D24" s="184"/>
+      <x:c r="E24" s="184"/>
+      <x:c r="F24" s="184"/>
+      <x:c r="G24" s="184"/>
+      <x:c r="H24" s="184"/>
+      <x:c r="I24" s="184"/>
+      <x:c r="J24" s="184"/>
+      <x:c r="K24" s="184"/>
+      <x:c r="L24" s="184"/>
+      <x:c r="M24" s="184"/>
+      <x:c r="N24" s="184"/>
+      <x:c r="O24" s="184"/>
+      <x:c r="P24" s="184"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="184"/>
+      <x:c r="B25" s="184"/>
+      <x:c r="C25" s="184"/>
+      <x:c r="D25" s="184"/>
+      <x:c r="E25" s="184"/>
+      <x:c r="F25" s="184"/>
+      <x:c r="G25" s="184"/>
+      <x:c r="H25" s="184"/>
+      <x:c r="I25" s="184"/>
+      <x:c r="J25" s="184"/>
+      <x:c r="K25" s="184"/>
+      <x:c r="L25" s="184"/>
+      <x:c r="M25" s="184"/>
+      <x:c r="N25" s="184"/>
+      <x:c r="O25" s="184"/>
+      <x:c r="P25" s="184"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="184"/>
+      <x:c r="B26" s="184"/>
+      <x:c r="C26" s="184"/>
+      <x:c r="D26" s="184"/>
+      <x:c r="E26" s="184"/>
+      <x:c r="F26" s="184"/>
+      <x:c r="G26" s="184"/>
+      <x:c r="H26" s="184"/>
+      <x:c r="I26" s="184"/>
+      <x:c r="J26" s="184"/>
+      <x:c r="K26" s="184"/>
+      <x:c r="L26" s="184"/>
+      <x:c r="M26" s="184"/>
+      <x:c r="N26" s="184"/>
+      <x:c r="O26" s="184"/>
+      <x:c r="P26" s="184"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="184"/>
+      <x:c r="B27" s="184"/>
+      <x:c r="C27" s="184"/>
+      <x:c r="D27" s="184"/>
+      <x:c r="E27" s="184"/>
+      <x:c r="F27" s="184"/>
+      <x:c r="G27" s="184"/>
+      <x:c r="H27" s="184"/>
+      <x:c r="I27" s="184"/>
+      <x:c r="J27" s="184"/>
+      <x:c r="K27" s="184"/>
+      <x:c r="L27" s="184"/>
+      <x:c r="M27" s="184"/>
+      <x:c r="N27" s="184"/>
+      <x:c r="O27" s="184"/>
+      <x:c r="P27" s="184"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="184"/>
+      <x:c r="B28" s="184"/>
+      <x:c r="C28" s="184"/>
+      <x:c r="D28" s="184"/>
+      <x:c r="E28" s="184"/>
+      <x:c r="F28" s="184"/>
+      <x:c r="G28" s="184"/>
+      <x:c r="H28" s="184"/>
+      <x:c r="I28" s="184"/>
+      <x:c r="J28" s="184"/>
+      <x:c r="K28" s="184"/>
+      <x:c r="L28" s="184"/>
+      <x:c r="M28" s="184"/>
+      <x:c r="N28" s="184"/>
+      <x:c r="O28" s="184"/>
+      <x:c r="P28" s="184"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="184"/>
+      <x:c r="B29" s="184"/>
+      <x:c r="C29" s="184"/>
+      <x:c r="D29" s="184"/>
+      <x:c r="E29" s="184"/>
+      <x:c r="F29" s="184"/>
+      <x:c r="G29" s="184"/>
+      <x:c r="H29" s="184"/>
+      <x:c r="I29" s="184"/>
+      <x:c r="J29" s="184"/>
+      <x:c r="K29" s="184"/>
+      <x:c r="L29" s="184"/>
+      <x:c r="M29" s="184"/>
+      <x:c r="N29" s="184"/>
+      <x:c r="O29" s="184"/>
+      <x:c r="P29" s="184"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="184"/>
+      <x:c r="B30" s="184"/>
+      <x:c r="C30" s="184"/>
+      <x:c r="D30" s="184"/>
+      <x:c r="E30" s="184"/>
+      <x:c r="F30" s="184"/>
+      <x:c r="G30" s="184"/>
+      <x:c r="H30" s="184"/>
+      <x:c r="I30" s="184"/>
+      <x:c r="J30" s="184"/>
+      <x:c r="K30" s="184"/>
+      <x:c r="L30" s="184"/>
+      <x:c r="M30" s="184"/>
+      <x:c r="N30" s="184"/>
+      <x:c r="O30" s="184"/>
+      <x:c r="P30" s="184"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="184"/>
+      <x:c r="B31" s="184"/>
+      <x:c r="C31" s="184"/>
+      <x:c r="D31" s="184"/>
+      <x:c r="E31" s="184"/>
+      <x:c r="F31" s="184"/>
+      <x:c r="G31" s="184"/>
+      <x:c r="H31" s="184"/>
+      <x:c r="I31" s="184"/>
+      <x:c r="J31" s="184"/>
+      <x:c r="K31" s="184"/>
+      <x:c r="L31" s="184"/>
+      <x:c r="M31" s="184"/>
+      <x:c r="N31" s="184"/>
+      <x:c r="O31" s="184"/>
+      <x:c r="P31" s="184"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="184"/>
+      <x:c r="B32" s="184"/>
+      <x:c r="C32" s="184"/>
+      <x:c r="D32" s="184"/>
+      <x:c r="E32" s="184"/>
+      <x:c r="F32" s="184"/>
+      <x:c r="G32" s="184"/>
+      <x:c r="H32" s="184"/>
+      <x:c r="I32" s="184"/>
+      <x:c r="J32" s="184"/>
+      <x:c r="K32" s="184"/>
+      <x:c r="L32" s="184"/>
+      <x:c r="M32" s="184"/>
+      <x:c r="N32" s="184"/>
+      <x:c r="O32" s="184"/>
+      <x:c r="P32" s="184"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="184"/>
+      <x:c r="B33" s="184"/>
+      <x:c r="C33" s="184"/>
+      <x:c r="D33" s="184"/>
+      <x:c r="E33" s="184"/>
+      <x:c r="F33" s="184"/>
+      <x:c r="G33" s="184"/>
+      <x:c r="H33" s="184"/>
+      <x:c r="I33" s="184"/>
+      <x:c r="J33" s="184"/>
+      <x:c r="K33" s="184"/>
+      <x:c r="L33" s="184"/>
+      <x:c r="M33" s="184"/>
+      <x:c r="N33" s="184"/>
+      <x:c r="O33" s="184"/>
+      <x:c r="P33" s="184"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="184"/>
+      <x:c r="B34" s="184"/>
+      <x:c r="C34" s="184"/>
+      <x:c r="D34" s="184"/>
+      <x:c r="E34" s="184"/>
+      <x:c r="F34" s="184"/>
+      <x:c r="G34" s="184"/>
+      <x:c r="H34" s="184"/>
+      <x:c r="I34" s="184"/>
+      <x:c r="J34" s="184"/>
+      <x:c r="K34" s="184"/>
+      <x:c r="L34" s="184"/>
+      <x:c r="M34" s="184"/>
+      <x:c r="N34" s="184"/>
+      <x:c r="O34" s="184"/>
+      <x:c r="P34" s="184"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="184"/>
+      <x:c r="B35" s="184"/>
+      <x:c r="C35" s="184"/>
+      <x:c r="D35" s="184"/>
+      <x:c r="E35" s="184"/>
+      <x:c r="F35" s="184"/>
+      <x:c r="G35" s="184"/>
+      <x:c r="H35" s="184"/>
+      <x:c r="I35" s="184"/>
+      <x:c r="J35" s="184"/>
+      <x:c r="K35" s="184"/>
+      <x:c r="L35" s="184"/>
+      <x:c r="M35" s="184"/>
+      <x:c r="N35" s="184"/>
+      <x:c r="O35" s="184"/>
+      <x:c r="P35" s="184"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="184"/>
+      <x:c r="B36" s="184"/>
+      <x:c r="C36" s="184"/>
+      <x:c r="D36" s="184"/>
+      <x:c r="E36" s="184"/>
+      <x:c r="F36" s="184"/>
+      <x:c r="G36" s="184"/>
+      <x:c r="H36" s="184"/>
+      <x:c r="I36" s="184"/>
+      <x:c r="J36" s="184"/>
+      <x:c r="K36" s="184"/>
+      <x:c r="L36" s="184"/>
+      <x:c r="M36" s="184"/>
+      <x:c r="N36" s="184"/>
+      <x:c r="O36" s="184"/>
+      <x:c r="P36" s="184"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="184"/>
+      <x:c r="B37" s="184"/>
+      <x:c r="C37" s="184"/>
+      <x:c r="D37" s="184"/>
+      <x:c r="E37" s="184"/>
+      <x:c r="F37" s="184"/>
+      <x:c r="G37" s="184"/>
+      <x:c r="H37" s="184"/>
+      <x:c r="I37" s="184"/>
+      <x:c r="J37" s="184"/>
+      <x:c r="K37" s="184"/>
+      <x:c r="L37" s="184"/>
+      <x:c r="M37" s="184"/>
+      <x:c r="N37" s="184"/>
+      <x:c r="O37" s="184"/>
+      <x:c r="P37" s="184"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="184"/>
+      <x:c r="B38" s="184"/>
+      <x:c r="C38" s="184"/>
+      <x:c r="D38" s="184"/>
+      <x:c r="E38" s="184"/>
+      <x:c r="F38" s="184"/>
+      <x:c r="G38" s="184"/>
+      <x:c r="H38" s="184"/>
+      <x:c r="I38" s="184"/>
+      <x:c r="J38" s="184"/>
+      <x:c r="K38" s="184"/>
+      <x:c r="L38" s="184"/>
+      <x:c r="M38" s="184"/>
+      <x:c r="N38" s="184"/>
+      <x:c r="O38" s="184"/>
+      <x:c r="P38" s="184"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="184"/>
+      <x:c r="B39" s="184"/>
+      <x:c r="C39" s="184"/>
+      <x:c r="D39" s="184"/>
+      <x:c r="E39" s="184"/>
+      <x:c r="F39" s="184"/>
+      <x:c r="G39" s="184"/>
+      <x:c r="H39" s="184"/>
+      <x:c r="I39" s="184"/>
+      <x:c r="J39" s="184"/>
+      <x:c r="K39" s="184"/>
+      <x:c r="L39" s="184"/>
+      <x:c r="M39" s="184"/>
+      <x:c r="N39" s="184"/>
+      <x:c r="O39" s="184"/>
+      <x:c r="P39" s="184"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="184"/>
+      <x:c r="B40" s="184"/>
+      <x:c r="C40" s="184"/>
+      <x:c r="D40" s="184"/>
+      <x:c r="E40" s="184"/>
+      <x:c r="F40" s="184"/>
+      <x:c r="G40" s="184"/>
+      <x:c r="H40" s="184"/>
+      <x:c r="I40" s="184"/>
+      <x:c r="J40" s="184"/>
+      <x:c r="K40" s="184"/>
+      <x:c r="L40" s="184"/>
+      <x:c r="M40" s="184"/>
+      <x:c r="N40" s="184"/>
+      <x:c r="O40" s="184"/>
+      <x:c r="P40" s="184"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="184"/>
+      <x:c r="B41" s="184"/>
+      <x:c r="C41" s="184"/>
+      <x:c r="D41" s="184"/>
+      <x:c r="E41" s="184"/>
+      <x:c r="F41" s="184"/>
+      <x:c r="G41" s="184"/>
+      <x:c r="H41" s="184"/>
+      <x:c r="I41" s="184"/>
+      <x:c r="J41" s="184"/>
+      <x:c r="K41" s="184"/>
+      <x:c r="L41" s="184"/>
+      <x:c r="M41" s="184"/>
+      <x:c r="N41" s="184"/>
+      <x:c r="O41" s="184"/>
+      <x:c r="P41" s="184"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="184"/>
+      <x:c r="B42" s="184"/>
+      <x:c r="C42" s="184"/>
+      <x:c r="D42" s="184"/>
+      <x:c r="E42" s="184"/>
+      <x:c r="F42" s="184"/>
+      <x:c r="G42" s="184"/>
+      <x:c r="H42" s="184"/>
+      <x:c r="I42" s="184"/>
+      <x:c r="J42" s="184"/>
+      <x:c r="K42" s="184"/>
+      <x:c r="L42" s="184"/>
+      <x:c r="M42" s="184"/>
+      <x:c r="N42" s="184"/>
+      <x:c r="O42" s="184"/>
+      <x:c r="P42" s="184"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="184"/>
+      <x:c r="B43" s="184"/>
+      <x:c r="C43" s="184"/>
+      <x:c r="D43" s="184"/>
+      <x:c r="E43" s="184"/>
+      <x:c r="F43" s="184"/>
+      <x:c r="G43" s="184"/>
+      <x:c r="H43" s="184"/>
+      <x:c r="I43" s="184"/>
+      <x:c r="J43" s="184"/>
+      <x:c r="K43" s="184"/>
+      <x:c r="L43" s="184"/>
+      <x:c r="M43" s="184"/>
+      <x:c r="N43" s="184"/>
+      <x:c r="O43" s="184"/>
+      <x:c r="P43" s="184"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="184"/>
+      <x:c r="B44" s="184"/>
+      <x:c r="C44" s="184"/>
+      <x:c r="D44" s="184"/>
+      <x:c r="E44" s="184"/>
+      <x:c r="F44" s="184"/>
+      <x:c r="G44" s="184"/>
+      <x:c r="H44" s="184"/>
+      <x:c r="I44" s="184"/>
+      <x:c r="J44" s="184"/>
+      <x:c r="K44" s="184"/>
+      <x:c r="L44" s="184"/>
+      <x:c r="M44" s="184"/>
+      <x:c r="N44" s="184"/>
+      <x:c r="O44" s="184"/>
+      <x:c r="P44" s="184"/>
+    </x:row>
+    <x:row r="45" ht="26" customHeight="1">
+      <x:c r="A45" s="780" t="str">
+        <x:v>주의: 본 대시보드는 공개 기록 기반 조사 현황입니다. 유행·검색·SNS 확산과 주가 반응의 인과관계를 단정하거나 매수를 권유하지 않습니다.</x:v>
+      </x:c>
+      <x:c r="B45" s="780"/>
+      <x:c r="C45" s="780"/>
+      <x:c r="D45" s="780"/>
+      <x:c r="E45" s="780"/>
+      <x:c r="F45" s="780"/>
+      <x:c r="G45" s="780"/>
+      <x:c r="H45" s="780"/>
+      <x:c r="I45" s="780"/>
+      <x:c r="J45" s="780"/>
+      <x:c r="K45" s="780"/>
+      <x:c r="L45" s="780"/>
+      <x:c r="M45" s="780"/>
+      <x:c r="N45" s="780"/>
+      <x:c r="O45" s="780"/>
+      <x:c r="P45" s="780"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="184"/>
+      <x:c r="B46" s="184"/>
+      <x:c r="C46" s="184"/>
+      <x:c r="D46" s="184"/>
+      <x:c r="E46" s="184"/>
+      <x:c r="F46" s="184"/>
+      <x:c r="G46" s="184"/>
+      <x:c r="H46" s="184"/>
+      <x:c r="I46" s="184"/>
+      <x:c r="J46" s="184"/>
+      <x:c r="K46" s="184"/>
+      <x:c r="L46" s="184"/>
+      <x:c r="M46" s="184"/>
+      <x:c r="N46" s="184"/>
+      <x:c r="O46" s="184"/>
+      <x:c r="P46" s="184"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="730" t="str">
+        <x:v>차트 계산 근거 — 01 유행이벤트 시트와 수식으로 연결</x:v>
+      </x:c>
+      <x:c r="B47" s="730"/>
+      <x:c r="C47" s="730"/>
+      <x:c r="D47" s="730"/>
+      <x:c r="E47" s="730"/>
+      <x:c r="F47" s="730"/>
+      <x:c r="G47" s="730"/>
+      <x:c r="H47" s="730"/>
+      <x:c r="I47" s="730"/>
+      <x:c r="J47" s="730"/>
+      <x:c r="K47" s="730"/>
+      <x:c r="L47" s="730"/>
+      <x:c r="M47" s="730"/>
+      <x:c r="N47" s="730"/>
+      <x:c r="O47" s="730"/>
+      <x:c r="P47" s="730"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="733" t="str">
+        <x:v>연도</x:v>
+      </x:c>
+      <x:c r="B48" s="733" t="str">
+        <x:v>사건 수</x:v>
+      </x:c>
+      <x:c r="C48" s="184"/>
+      <x:c r="D48" s="733" t="str">
+        <x:v>대분류</x:v>
+      </x:c>
+      <x:c r="E48" s="733" t="str">
+        <x:v>전체 사건</x:v>
+      </x:c>
+      <x:c r="F48" s="733" t="str">
+        <x:v>주가 연결</x:v>
+      </x:c>
+      <x:c r="G48" s="733" t="str">
+        <x:v>연결률</x:v>
+      </x:c>
+      <x:c r="H48" s="184"/>
+      <x:c r="I48" s="733" t="str">
+        <x:v>주가 연결 상태</x:v>
+      </x:c>
+      <x:c r="J48" s="733" t="str">
+        <x:v>사건 수</x:v>
+      </x:c>
+      <x:c r="K48" s="733" t="str">
+        <x:v>대분류</x:v>
+      </x:c>
+      <x:c r="L48" s="733" t="str">
+        <x:v>주가 연결률</x:v>
+      </x:c>
+      <x:c r="M48" s="184"/>
+      <x:c r="N48" s="747" t="str">
+        <x:v>해석 주의</x:v>
+      </x:c>
+      <x:c r="O48" s="747"/>
+      <x:c r="P48" s="747"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="742" t="str">
+        <x:v>2009</x:v>
+      </x:c>
+      <x:c r="B49" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A49)</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C49" s="184"/>
+      <x:c r="D49" s="737" t="str">
+        <x:v>콘텐츠·엔터</x:v>
+      </x:c>
+      <x:c r="E49" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D49)</x:f>
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="F49" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D49,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G49" s="744" t="n">
+        <x:f>IFERROR(F49/E49,0)</x:f>
+        <x:v>0.23595505617977527</x:v>
+      </x:c>
+      <x:c r="H49" s="184"/>
+      <x:c r="I49" s="737" t="str">
+        <x:v>주가 반응 기록 있음</x:v>
+      </x:c>
+      <x:c r="J49" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$I$6:$I$303,I49)</x:f>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="K49" s="737" t="str">
+        <x:f>D49</x:f>
+        <x:v>콘텐츠·엔터</x:v>
+      </x:c>
+      <x:c r="L49" s="744" t="n">
+        <x:f>G49</x:f>
+        <x:v>0.23595505617977527</x:v>
+      </x:c>
+      <x:c r="M49" s="184"/>
+      <x:c r="N49" s="768" t="str">
+        <x:v>• 연결률은 “주가 영향 확률”이 아니라 현재 원장에서 가격 근거까지 확보된 비중입니다.
+• 금융·시장현상은 5건뿐이므로 100% 수치를 일반화하면 안 됩니다.
+• 2026년은 진행 중인 연도라 과거 완결 연도와 직접 비교할 때 주의합니다.</x:v>
+      </x:c>
+      <x:c r="O49" s="769"/>
+      <x:c r="P49" s="770"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="742" t="str">
+        <x:v>2010</x:v>
+      </x:c>
+      <x:c r="B50" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A50)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C50" s="184"/>
+      <x:c r="D50" s="737" t="str">
+        <x:v>식품·음료</x:v>
+      </x:c>
+      <x:c r="E50" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D50)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F50" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D50,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G50" s="744" t="n">
+        <x:f>IFERROR(F50/E50,0)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H50" s="184"/>
+      <x:c r="I50" s="737" t="str">
+        <x:v>주가 미확인·연결 전</x:v>
+      </x:c>
+      <x:c r="J50" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$I$6:$I$303,I50)</x:f>
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="K50" s="737" t="str">
+        <x:f>D50</x:f>
+        <x:v>식품·음료</x:v>
+      </x:c>
+      <x:c r="L50" s="744" t="n">
+        <x:f>G50</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="M50" s="184"/>
+      <x:c r="N50" s="771"/>
+      <x:c r="O50" s="772"/>
+      <x:c r="P50" s="773"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="742" t="str">
+        <x:v>2011</x:v>
+      </x:c>
+      <x:c r="B51" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A51)</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C51" s="184"/>
+      <x:c r="D51" s="737" t="str">
+        <x:v>디지털·플랫폼</x:v>
+      </x:c>
+      <x:c r="E51" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D51)</x:f>
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="F51" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D51,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G51" s="744" t="n">
+        <x:f>IFERROR(F51/E51,0)</x:f>
+        <x:v>0.11627906976744186</x:v>
+      </x:c>
+      <x:c r="H51" s="184"/>
+      <x:c r="I51" s="184"/>
+      <x:c r="J51" s="184"/>
+      <x:c r="K51" s="737" t="str">
+        <x:f>D51</x:f>
+        <x:v>디지털·플랫폼</x:v>
+      </x:c>
+      <x:c r="L51" s="744" t="n">
+        <x:f>G51</x:f>
+        <x:v>0.11627906976744186</x:v>
+      </x:c>
+      <x:c r="M51" s="184"/>
+      <x:c r="N51" s="771"/>
+      <x:c r="O51" s="772"/>
+      <x:c r="P51" s="773"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="742" t="str">
+        <x:v>2012</x:v>
+      </x:c>
+      <x:c r="B52" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A52)</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C52" s="184"/>
+      <x:c r="D52" s="737" t="str">
+        <x:v>게임·e스포츠</x:v>
+      </x:c>
+      <x:c r="E52" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D52)</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F52" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D52,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G52" s="744" t="n">
+        <x:f>IFERROR(F52/E52,0)</x:f>
+        <x:v>0.08695652173913043</x:v>
+      </x:c>
+      <x:c r="H52" s="184"/>
+      <x:c r="I52" s="184"/>
+      <x:c r="J52" s="184"/>
+      <x:c r="K52" s="737" t="str">
+        <x:f>D52</x:f>
+        <x:v>게임·e스포츠</x:v>
+      </x:c>
+      <x:c r="L52" s="744" t="n">
+        <x:f>G52</x:f>
+        <x:v>0.08695652173913043</x:v>
+      </x:c>
+      <x:c r="M52" s="184"/>
+      <x:c r="N52" s="771"/>
+      <x:c r="O52" s="772"/>
+      <x:c r="P52" s="773"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="742" t="str">
+        <x:v>2013</x:v>
+      </x:c>
+      <x:c r="B53" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A53)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C53" s="184"/>
+      <x:c r="D53" s="737" t="str">
+        <x:v>패션·뷰티</x:v>
+      </x:c>
+      <x:c r="E53" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D53)</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="F53" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D53,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G53" s="744" t="n">
+        <x:f>IFERROR(F53/E53,0)</x:f>
+        <x:v>0.15789473684210525</x:v>
+      </x:c>
+      <x:c r="H53" s="184"/>
+      <x:c r="I53" s="184"/>
+      <x:c r="J53" s="184"/>
+      <x:c r="K53" s="737" t="str">
+        <x:f>D53</x:f>
+        <x:v>패션·뷰티</x:v>
+      </x:c>
+      <x:c r="L53" s="744" t="n">
+        <x:f>G53</x:f>
+        <x:v>0.15789473684210525</x:v>
+      </x:c>
+      <x:c r="M53" s="184"/>
+      <x:c r="N53" s="771"/>
+      <x:c r="O53" s="772"/>
+      <x:c r="P53" s="773"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="742" t="str">
+        <x:v>2014</x:v>
+      </x:c>
+      <x:c r="B54" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A54)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C54" s="184"/>
+      <x:c r="D54" s="737" t="str">
+        <x:v>생활·소비</x:v>
+      </x:c>
+      <x:c r="E54" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D54)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F54" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D54,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G54" s="744" t="n">
+        <x:f>IFERROR(F54/E54,0)</x:f>
+        <x:v>0.3125</x:v>
+      </x:c>
+      <x:c r="H54" s="184"/>
+      <x:c r="I54" s="184"/>
+      <x:c r="J54" s="184"/>
+      <x:c r="K54" s="737" t="str">
+        <x:f>D54</x:f>
+        <x:v>생활·소비</x:v>
+      </x:c>
+      <x:c r="L54" s="744" t="n">
+        <x:f>G54</x:f>
+        <x:v>0.3125</x:v>
+      </x:c>
+      <x:c r="M54" s="184"/>
+      <x:c r="N54" s="771"/>
+      <x:c r="O54" s="772"/>
+      <x:c r="P54" s="773"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="742" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="B55" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A55)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C55" s="184"/>
+      <x:c r="D55" s="737" t="str">
+        <x:v>사회·온라인문화</x:v>
+      </x:c>
+      <x:c r="E55" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D55)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F55" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D55,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G7" s="111" t="str">
-        <x:v>유행 존재와 확산 이유를 먼저 확인</x:v>
-      </x:c>
-      <x:c r="H7" s="111"/>
-      <x:c r="I7" s="111"/>
-      <x:c r="J7" s="111"/>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="113" t="str">
-        <x:v>02 종목반응</x:v>
-      </x:c>
-      <x:c r="B8" s="111" t="str">
-        <x:v>연도 내림차순이며 사건과 동일한 대분류·소분류 적용</x:v>
-      </x:c>
-      <x:c r="C8" s="111"/>
-      <x:c r="D8" s="111"/>
-      <x:c r="E8" s="111"/>
-      <x:c r="F8" s="116" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G8" s="111" t="str">
-        <x:v>주가 미확인은 “영향 없음”이 아니라 후속 조사 대기 상태</x:v>
-      </x:c>
-      <x:c r="H8" s="111"/>
-      <x:c r="I8" s="111"/>
-      <x:c r="J8" s="111"/>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="113" t="str">
-        <x:v>03 출처</x:v>
-      </x:c>
-      <x:c r="B9" s="111" t="str">
-        <x:v>확인 가능한 발행일 기준 최신순, 출처ID는 고정</x:v>
-      </x:c>
-      <x:c r="C9" s="111"/>
-      <x:c r="D9" s="111"/>
-      <x:c r="E9" s="111"/>
-      <x:c r="F9" s="116" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G9" s="111" t="str">
-        <x:v>주가 반응 표에는 실제 가격·일자 근거가 있는 사례만 유지</x:v>
-      </x:c>
-      <x:c r="H9" s="111"/>
-      <x:c r="I9" s="111"/>
-      <x:c r="J9" s="111"/>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="113" t="str">
-        <x:v>04 판정기준</x:v>
-      </x:c>
-      <x:c r="B10" s="111" t="str">
-        <x:v>포함·연결 기준과 9개 대분류 체계를 함께 확인</x:v>
-      </x:c>
-      <x:c r="C10" s="111"/>
-      <x:c r="D10" s="111"/>
-      <x:c r="E10" s="111"/>
-      <x:c r="F10" s="116" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G10" s="111" t="str">
-        <x:v>같은 시기 실적·공시 등 동시 재료를 반드시 분리</x:v>
-      </x:c>
-      <x:c r="H10" s="111"/>
-      <x:c r="I10" s="111"/>
-      <x:c r="J10" s="111"/>
-    </x:row>
-    <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="113" t="str">
-        <x:v>포함</x:v>
-      </x:c>
-      <x:c r="B11" s="111" t="str">
-        <x:v>식품·음료, 콘텐츠·엔터, 디지털·플랫폼, 게임, 패션·뷰티, 생활, 스포츠, 온라인문화, 시장현상</x:v>
-      </x:c>
-      <x:c r="C11" s="111"/>
-      <x:c r="D11" s="111"/>
-      <x:c r="E11" s="111"/>
-      <x:c r="F11" s="116" t="str">
+      <x:c r="G55" s="744" t="n">
+        <x:f>IFERROR(F55/E55,0)</x:f>
+        <x:v>0.07142857142857142</x:v>
+      </x:c>
+      <x:c r="H55" s="184"/>
+      <x:c r="I55" s="184"/>
+      <x:c r="J55" s="184"/>
+      <x:c r="K55" s="737" t="str">
+        <x:f>D55</x:f>
+        <x:v>사회·온라인문화</x:v>
+      </x:c>
+      <x:c r="L55" s="744" t="n">
+        <x:f>G55</x:f>
+        <x:v>0.07142857142857142</x:v>
+      </x:c>
+      <x:c r="M55" s="184"/>
+      <x:c r="N55" s="771"/>
+      <x:c r="O55" s="772"/>
+      <x:c r="P55" s="773"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="742" t="str">
+        <x:v>2016</x:v>
+      </x:c>
+      <x:c r="B56" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A56)</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C56" s="184"/>
+      <x:c r="D56" s="737" t="str">
+        <x:v>스포츠·건강</x:v>
+      </x:c>
+      <x:c r="E56" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D56)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F56" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D56,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G56" s="744" t="n">
+        <x:f>IFERROR(F56/E56,0)</x:f>
+        <x:v>0.6923076923076923</x:v>
+      </x:c>
+      <x:c r="H56" s="184"/>
+      <x:c r="I56" s="184"/>
+      <x:c r="J56" s="184"/>
+      <x:c r="K56" s="737" t="str">
+        <x:f>D56</x:f>
+        <x:v>스포츠·건강</x:v>
+      </x:c>
+      <x:c r="L56" s="744" t="n">
+        <x:f>G56</x:f>
+        <x:v>0.6923076923076923</x:v>
+      </x:c>
+      <x:c r="M56" s="184"/>
+      <x:c r="N56" s="771"/>
+      <x:c r="O56" s="772"/>
+      <x:c r="P56" s="773"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="742" t="str">
+        <x:v>2017</x:v>
+      </x:c>
+      <x:c r="B57" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A57)</x:f>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C57" s="184"/>
+      <x:c r="D57" s="737" t="str">
+        <x:v>금융·시장현상</x:v>
+      </x:c>
+      <x:c r="E57" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$C$6:$C$303,D57)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G11" s="111" t="str">
-        <x:v>유행은 매수 신호가 아니라 기업 조사의 출발점</x:v>
-      </x:c>
-      <x:c r="H11" s="111"/>
-      <x:c r="I11" s="111"/>
-      <x:c r="J11" s="111"/>
-    </x:row>
-    <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="113" t="str">
-        <x:v>제외</x:v>
-      </x:c>
-      <x:c r="B12" s="111" t="str">
-        <x:v>정치인·선거·공약·정책·정부사업 테마</x:v>
-      </x:c>
-      <x:c r="C12" s="111"/>
-      <x:c r="D12" s="111"/>
-      <x:c r="E12" s="111"/>
-      <x:c r="F12" s="116" t="str">
-        <x:v>한계</x:v>
-      </x:c>
-      <x:c r="G12" s="111" t="str">
-        <x:v>삭제 게시물·비공개 커뮤니티 때문에 “완전 전수”는 불가능</x:v>
-      </x:c>
-      <x:c r="H12" s="111"/>
-      <x:c r="I12" s="111"/>
-      <x:c r="J12" s="111"/>
-    </x:row>
-    <x:row r="14" ht="34" customHeight="1">
-      <x:c r="A14" s="118" t="str">
-        <x:v>연도별 유행 사건 수 — 최신 연도부터 확인</x:v>
-      </x:c>
-      <x:c r="B14" s="118"/>
-      <x:c r="C14" s="118"/>
-      <x:c r="D14" s="118"/>
-      <x:c r="E14" s="118"/>
-      <x:c r="F14" s="118"/>
-      <x:c r="G14" s="118"/>
-      <x:c r="H14" s="118"/>
-      <x:c r="I14" s="118"/>
-      <x:c r="J14" s="118"/>
-    </x:row>
-    <x:row r="16" ht="28" customHeight="1">
-      <x:c r="A16" s="121" t="n">
+      <x:c r="F57" s="743" t="n">
+        <x:f>COUNTIFS('01_유행이벤트'!$C$6:$C$303,D57,'01_유행이벤트'!$I$6:$I$303,"주가 반응 기록 있음")</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G57" s="744" t="n">
+        <x:f>IFERROR(F57/E57,0)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H57" s="184"/>
+      <x:c r="I57" s="184"/>
+      <x:c r="J57" s="184"/>
+      <x:c r="K57" s="737" t="str">
+        <x:f>D57</x:f>
+        <x:v>금융·시장현상</x:v>
+      </x:c>
+      <x:c r="L57" s="744" t="n">
+        <x:f>G57</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M57" s="184"/>
+      <x:c r="N57" s="774"/>
+      <x:c r="O57" s="775"/>
+      <x:c r="P57" s="776"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="742" t="str">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="B58" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A58)</x:f>
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C58" s="184"/>
+      <x:c r="D58" s="184"/>
+      <x:c r="E58" s="184"/>
+      <x:c r="F58" s="184"/>
+      <x:c r="G58" s="184"/>
+      <x:c r="H58" s="184"/>
+      <x:c r="I58" s="184"/>
+      <x:c r="J58" s="184"/>
+      <x:c r="K58" s="184"/>
+      <x:c r="L58" s="184"/>
+      <x:c r="M58" s="184"/>
+      <x:c r="N58" s="184"/>
+      <x:c r="O58" s="184"/>
+      <x:c r="P58" s="184"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="742" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="B59" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A59)</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C59" s="184"/>
+      <x:c r="D59" s="184"/>
+      <x:c r="E59" s="184"/>
+      <x:c r="F59" s="184"/>
+      <x:c r="G59" s="184"/>
+      <x:c r="H59" s="184"/>
+      <x:c r="I59" s="184"/>
+      <x:c r="J59" s="184"/>
+      <x:c r="K59" s="184"/>
+      <x:c r="L59" s="184"/>
+      <x:c r="M59" s="184"/>
+      <x:c r="N59" s="184"/>
+      <x:c r="O59" s="184"/>
+      <x:c r="P59" s="184"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="742" t="str">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="B60" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A60)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C60" s="184"/>
+      <x:c r="D60" s="184"/>
+      <x:c r="E60" s="184"/>
+      <x:c r="F60" s="184"/>
+      <x:c r="G60" s="184"/>
+      <x:c r="H60" s="184"/>
+      <x:c r="I60" s="184"/>
+      <x:c r="J60" s="184"/>
+      <x:c r="K60" s="184"/>
+      <x:c r="L60" s="184"/>
+      <x:c r="M60" s="184"/>
+      <x:c r="N60" s="184"/>
+      <x:c r="O60" s="184"/>
+      <x:c r="P60" s="184"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="742" t="str">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="B61" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A61)</x:f>
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C61" s="184"/>
+      <x:c r="D61" s="184"/>
+      <x:c r="E61" s="184"/>
+      <x:c r="F61" s="184"/>
+      <x:c r="G61" s="184"/>
+      <x:c r="H61" s="184"/>
+      <x:c r="I61" s="184"/>
+      <x:c r="J61" s="184"/>
+      <x:c r="K61" s="184"/>
+      <x:c r="L61" s="184"/>
+      <x:c r="M61" s="184"/>
+      <x:c r="N61" s="184"/>
+      <x:c r="O61" s="184"/>
+      <x:c r="P61" s="184"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="742" t="str">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="B62" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A62)</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C62" s="184"/>
+      <x:c r="D62" s="184"/>
+      <x:c r="E62" s="184"/>
+      <x:c r="F62" s="184"/>
+      <x:c r="G62" s="184"/>
+      <x:c r="H62" s="184"/>
+      <x:c r="I62" s="184"/>
+      <x:c r="J62" s="184"/>
+      <x:c r="K62" s="184"/>
+      <x:c r="L62" s="184"/>
+      <x:c r="M62" s="184"/>
+      <x:c r="N62" s="184"/>
+      <x:c r="O62" s="184"/>
+      <x:c r="P62" s="184"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="742" t="str">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="B63" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A63)</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C63" s="184"/>
+      <x:c r="D63" s="184"/>
+      <x:c r="E63" s="184"/>
+      <x:c r="F63" s="184"/>
+      <x:c r="G63" s="184"/>
+      <x:c r="H63" s="184"/>
+      <x:c r="I63" s="184"/>
+      <x:c r="J63" s="184"/>
+      <x:c r="K63" s="184"/>
+      <x:c r="L63" s="184"/>
+      <x:c r="M63" s="184"/>
+      <x:c r="N63" s="184"/>
+      <x:c r="O63" s="184"/>
+      <x:c r="P63" s="184"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="742" t="str">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="B64" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A64)</x:f>
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C64" s="184"/>
+      <x:c r="D64" s="184"/>
+      <x:c r="E64" s="184"/>
+      <x:c r="F64" s="184"/>
+      <x:c r="G64" s="184"/>
+      <x:c r="H64" s="184"/>
+      <x:c r="I64" s="184"/>
+      <x:c r="J64" s="184"/>
+      <x:c r="K64" s="184"/>
+      <x:c r="L64" s="184"/>
+      <x:c r="M64" s="184"/>
+      <x:c r="N64" s="184"/>
+      <x:c r="O64" s="184"/>
+      <x:c r="P64" s="184"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="742" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="B65" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A65)</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C65" s="184"/>
+      <x:c r="D65" s="184"/>
+      <x:c r="E65" s="184"/>
+      <x:c r="F65" s="184"/>
+      <x:c r="G65" s="184"/>
+      <x:c r="H65" s="184"/>
+      <x:c r="I65" s="184"/>
+      <x:c r="J65" s="184"/>
+      <x:c r="K65" s="184"/>
+      <x:c r="L65" s="184"/>
+      <x:c r="M65" s="184"/>
+      <x:c r="N65" s="184"/>
+      <x:c r="O65" s="184"/>
+      <x:c r="P65" s="184"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="742" t="str">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="B16" s="121" t="n">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="C16" s="121" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="D16" s="121" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="E16" s="121" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="F16" s="121" t="n">
-        <x:v>2021</x:v>
-      </x:c>
-      <x:c r="G16" s="121" t="n">
-        <x:v>2020</x:v>
-      </x:c>
-      <x:c r="H16" s="121" t="n">
-        <x:v>2019</x:v>
-      </x:c>
-      <x:c r="I16" s="121" t="n">
-        <x:v>2018</x:v>
-      </x:c>
-      <x:c r="J16"/>
-    </x:row>
-    <x:row r="17" ht="28" customHeight="1">
-      <x:c r="A17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A16)</x:f>
+      <x:c r="B66" s="743" t="n">
+        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A66)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,B16)</x:f>
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="C17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,C16)</x:f>
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,D16)</x:f>
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,E16)</x:f>
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="F17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,F16)</x:f>
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="G17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,G16)</x:f>
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,H16)</x:f>
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I17" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,I16)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="J17"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="121" t="n">
-        <x:v>2017</x:v>
-      </x:c>
-      <x:c r="B19" s="121" t="n">
-        <x:v>2016</x:v>
-      </x:c>
-      <x:c r="C19" s="121" t="n">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="D19" s="121" t="n">
-        <x:v>2014</x:v>
-      </x:c>
-      <x:c r="E19" s="121" t="n">
-        <x:v>2013</x:v>
-      </x:c>
-      <x:c r="F19" s="121" t="n">
-        <x:v>2012</x:v>
-      </x:c>
-      <x:c r="G19" s="121" t="n">
-        <x:v>2011</x:v>
-      </x:c>
-      <x:c r="H19" s="121" t="n">
-        <x:v>2010</x:v>
-      </x:c>
-      <x:c r="I19" s="121" t="n">
-        <x:v>2009</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,A19)</x:f>
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,B19)</x:f>
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,C19)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,D19)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,E19)</x:f>
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,F19)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,G19)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="H20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,H19)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="I20" s="125" t="n">
-        <x:f>COUNTIF('01_유행이벤트'!$B$6:$B$303,I19)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="34" customHeight="1">
-      <x:c r="A22" s="129" t="str">
-        <x:v>주의: 이 원장은 유행·검색·플랫폼 확산의 조사 자료이며 투자 추천이 아닙니다. 인과관계는 각 출처가 확인하는 범위까지만 표시합니다.</x:v>
-      </x:c>
-      <x:c r="B22" s="129"/>
-      <x:c r="C22" s="129"/>
-      <x:c r="D22" s="129"/>
-      <x:c r="E22" s="129"/>
-      <x:c r="F22" s="129"/>
-      <x:c r="G22" s="129"/>
-      <x:c r="H22" s="129"/>
-      <x:c r="I22" s="129"/>
-      <x:c r="J22" s="129"/>
+      <x:c r="C66" s="184"/>
+      <x:c r="D66" s="184"/>
+      <x:c r="E66" s="184"/>
+      <x:c r="F66" s="184"/>
+      <x:c r="G66" s="184"/>
+      <x:c r="H66" s="184"/>
+      <x:c r="I66" s="184"/>
+      <x:c r="J66" s="184"/>
+      <x:c r="K66" s="184"/>
+      <x:c r="L66" s="184"/>
+      <x:c r="M66" s="184"/>
+      <x:c r="N66" s="184"/>
+      <x:c r="O66" s="184"/>
+      <x:c r="P66" s="184"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="184"/>
+      <x:c r="B67" s="184"/>
+      <x:c r="C67" s="184"/>
+      <x:c r="D67" s="184"/>
+      <x:c r="E67" s="184"/>
+      <x:c r="F67" s="184"/>
+      <x:c r="G67" s="184"/>
+      <x:c r="H67" s="184"/>
+      <x:c r="I67" s="184"/>
+      <x:c r="J67" s="184"/>
+      <x:c r="K67" s="184"/>
+      <x:c r="L67" s="184"/>
+      <x:c r="M67" s="184"/>
+      <x:c r="N67" s="184"/>
+      <x:c r="O67" s="184"/>
+      <x:c r="P67" s="184"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A6:E6"/>
-    <x:mergeCell ref="F6:J6"/>
-    <x:mergeCell ref="A22:J22"/>
-    <x:mergeCell ref="B7:E7"/>
-    <x:mergeCell ref="G7:J7"/>
-    <x:mergeCell ref="B8:E8"/>
-    <x:mergeCell ref="G8:J8"/>
-    <x:mergeCell ref="B9:E9"/>
-    <x:mergeCell ref="G9:J9"/>
-    <x:mergeCell ref="B10:E10"/>
-    <x:mergeCell ref="G10:J10"/>
-    <x:mergeCell ref="B11:E11"/>
-    <x:mergeCell ref="G11:J11"/>
-    <x:mergeCell ref="B12:E12"/>
-    <x:mergeCell ref="G12:J12"/>
-    <x:mergeCell ref="A2:J2"/>
-    <x:mergeCell ref="A14:J14"/>
+    <x:mergeCell ref="A1:P1"/>
+    <x:mergeCell ref="A2:P2"/>
+    <x:mergeCell ref="A3:P3"/>
+    <x:mergeCell ref="A5:C5"/>
+    <x:mergeCell ref="A6:C7"/>
+    <x:mergeCell ref="A8:C8"/>
+    <x:mergeCell ref="D5:F5"/>
+    <x:mergeCell ref="D6:F7"/>
+    <x:mergeCell ref="D8:F8"/>
+    <x:mergeCell ref="G5:I5"/>
+    <x:mergeCell ref="G6:I7"/>
+    <x:mergeCell ref="G8:I8"/>
+    <x:mergeCell ref="J5:L5"/>
+    <x:mergeCell ref="J6:L7"/>
+    <x:mergeCell ref="J8:L8"/>
+    <x:mergeCell ref="M5:P5"/>
+    <x:mergeCell ref="M6:P7"/>
+    <x:mergeCell ref="M8:P8"/>
+    <x:mergeCell ref="A10:P10"/>
+    <x:mergeCell ref="A11:E12"/>
+    <x:mergeCell ref="F11:J12"/>
+    <x:mergeCell ref="K11:P12"/>
+    <x:mergeCell ref="A47:P47"/>
+    <x:mergeCell ref="N48:P48"/>
+    <x:mergeCell ref="N49:P57"/>
+    <x:mergeCell ref="A45:P45"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8cbb35c80f475e"/>
 </x:worksheet>
 </file>
 
@@ -13606,7 +16941,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d6ca49ce79046b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ed60b71aef04103"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26376,7 +29711,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd59045c1004405b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3e72239bf7a4332"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>